<commit_message>
Started entering Sept 2023 Sulfide Sample IDs and Dilutions
</commit_message>
<xml_diff>
--- a/Porewater/Sulfide/Synoptic_CB/2023/Raw Data/COMPASS_Synoptic_H2S_Sept2023.xlsx
+++ b/Porewater/Sulfide/Synoptic_CB/2023/Raw Data/COMPASS_Synoptic_H2S_Sept2023.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26130"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\Biogeochemistry\People\Wilson (Steph)\Data\MicroPlate Data\Sulfide\Data\2023\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://sinet-my.sharepoint.com/personal/readz_si_edu1/Documents/synoptic-discrete-data/Porewater/Sulfide/Synoptic_CB/2023/Raw Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B0E3FFA-5A27-4C59-B6BE-4DCE142CEFF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="135" documentId="13_ncr:1_{4B0E3FFA-5A27-4C59-B6BE-4DCE142CEFF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0E1987D3-9DFD-4B7A-B46C-21469AF698D2}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="15000" xr2:uid="{BFEEA0A9-30A3-45FE-8475-2FD233249056}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{BFEEA0A9-30A3-45FE-8475-2FD233249056}"/>
   </bookViews>
   <sheets>
     <sheet name="STDs" sheetId="1" r:id="rId1"/>
@@ -22,9 +22,6 @@
     <sheet name="Plate6" sheetId="7" r:id="rId7"/>
     <sheet name="Plate7" sheetId="8" r:id="rId8"/>
   </sheets>
-  <externalReferences>
-    <externalReference r:id="rId9"/>
-  </externalReferences>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -46,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="392" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="537" uniqueCount="79">
   <si>
     <t>Plate 1</t>
   </si>
@@ -136,6 +133,153 @@
   </si>
   <si>
     <t>Dilutions</t>
+  </si>
+  <si>
+    <t>GCW_UP_LysA_20cm</t>
+  </si>
+  <si>
+    <t>GCW_TR_LysA_20cm</t>
+  </si>
+  <si>
+    <t>GCW_TR_LysA_45cm</t>
+  </si>
+  <si>
+    <t>GCW_TR_LysB_10cm</t>
+  </si>
+  <si>
+    <t>GCW_TR_LysB_20cm</t>
+  </si>
+  <si>
+    <t>GCW_TR_LysB_45cm</t>
+  </si>
+  <si>
+    <t>GCW_TR_LysC_10cm</t>
+  </si>
+  <si>
+    <t>GCW_TR_LysC_20cm</t>
+  </si>
+  <si>
+    <t>GCW_TR_LysC_45cm</t>
+  </si>
+  <si>
+    <t>GCW_WC_LysA_10cm</t>
+  </si>
+  <si>
+    <t>GCW_WC_LysA_20cm</t>
+  </si>
+  <si>
+    <t>GCW_WC_LysA_45cm</t>
+  </si>
+  <si>
+    <t>GCW_WC_LysB_10cm</t>
+  </si>
+  <si>
+    <t>GCW_WC_LysB_10cm_dup</t>
+  </si>
+  <si>
+    <t>GCW_WC_LysB_20cm</t>
+  </si>
+  <si>
+    <t>GCW_WC_LysB_20cm_spk</t>
+  </si>
+  <si>
+    <t>GCW_WC_LysB_45cm</t>
+  </si>
+  <si>
+    <t>GCW_WC_LysC_10cm</t>
+  </si>
+  <si>
+    <t>GCW_WC_LysC_20cm</t>
+  </si>
+  <si>
+    <t>GCW_WC_LysC_45cm</t>
+  </si>
+  <si>
+    <t>GCW_SW_A</t>
+  </si>
+  <si>
+    <t>GCW_SW_B</t>
+  </si>
+  <si>
+    <t>GCW_SW_C</t>
+  </si>
+  <si>
+    <t>MSM_UP_LysA_45cm</t>
+  </si>
+  <si>
+    <t>MSM_UP_LysB_10cm</t>
+  </si>
+  <si>
+    <t>MSM_UP_LysB_45cm</t>
+  </si>
+  <si>
+    <t>MSM_UP_LysC_10cm</t>
+  </si>
+  <si>
+    <t>MSM_UP_LysC_20cm</t>
+  </si>
+  <si>
+    <t>MSM_UP_LysC_45cm</t>
+  </si>
+  <si>
+    <t>MSM_TR_LysA_10cm</t>
+  </si>
+  <si>
+    <t>MSM_TR_LysA_20cm</t>
+  </si>
+  <si>
+    <t>MSM_TR_LysA_45cm</t>
+  </si>
+  <si>
+    <t>MSM_TR_LysB_10cm</t>
+  </si>
+  <si>
+    <t>MSM_TR_LysB_20cm</t>
+  </si>
+  <si>
+    <t>MSM_TR_LysB_45cm</t>
+  </si>
+  <si>
+    <t>MSM_TR_LysC_10cm</t>
+  </si>
+  <si>
+    <t>MSM_TR_LysC_20cm</t>
+  </si>
+  <si>
+    <t>MSM_TR_LysC_20cm_dup</t>
+  </si>
+  <si>
+    <t>MSM_TR_LysC_45cm</t>
+  </si>
+  <si>
+    <t>MSM_TR_LysC_45cm_spk</t>
+  </si>
+  <si>
+    <t>MSM_WC_LysA_10cm</t>
+  </si>
+  <si>
+    <t>MSM_WC_LysB_45cm</t>
+  </si>
+  <si>
+    <t>MSM_WC_LysC_10cm</t>
+  </si>
+  <si>
+    <t>MSM_WC_LysA_20cm</t>
+  </si>
+  <si>
+    <t>MSM_WC_LysA_45cm</t>
+  </si>
+  <si>
+    <t>MSM_WC_LysB_10cm</t>
+  </si>
+  <si>
+    <t>MSM_WC_LysB_20cm</t>
+  </si>
+  <si>
+    <t>MSM_WC_LysC_20cm</t>
+  </si>
+  <si>
+    <t>MSM_WC_LysC_45cm</t>
   </si>
 </sst>
 </file>
@@ -7153,530 +7297,10 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <sheetNames>
-      <sheetName val="STDs"/>
-      <sheetName val="Plate1"/>
-      <sheetName val="Plate2"/>
-      <sheetName val="Plate3"/>
-      <sheetName val="Plate4"/>
-      <sheetName val="Plate5"/>
-      <sheetName val="Plate6"/>
-      <sheetName val="Plate7"/>
-      <sheetName val="Plate8"/>
-      <sheetName val="Sheet4"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0">
-        <row r="2">
-          <cell r="B2" t="str">
-            <v>Avg Abs</v>
-          </cell>
-        </row>
-        <row r="3">
-          <cell r="A3">
-            <v>0</v>
-          </cell>
-          <cell r="B3">
-            <v>5.0666666666666665E-2</v>
-          </cell>
-        </row>
-        <row r="4">
-          <cell r="A4">
-            <v>5</v>
-          </cell>
-          <cell r="B4">
-            <v>0.13566666666666669</v>
-          </cell>
-        </row>
-        <row r="5">
-          <cell r="A5">
-            <v>12.5</v>
-          </cell>
-          <cell r="B5">
-            <v>0.23949999999999999</v>
-          </cell>
-        </row>
-        <row r="6">
-          <cell r="A6">
-            <v>25</v>
-          </cell>
-          <cell r="B6">
-            <v>0.42399999999999999</v>
-          </cell>
-        </row>
-        <row r="7">
-          <cell r="A7">
-            <v>50</v>
-          </cell>
-          <cell r="B7">
-            <v>0.76</v>
-          </cell>
-        </row>
-        <row r="8">
-          <cell r="A8">
-            <v>100</v>
-          </cell>
-          <cell r="B8">
-            <v>1.232</v>
-          </cell>
-        </row>
-        <row r="13">
-          <cell r="B13" t="str">
-            <v>Avg Abs</v>
-          </cell>
-        </row>
-        <row r="14">
-          <cell r="A14">
-            <v>0</v>
-          </cell>
-          <cell r="B14">
-            <v>4.933333333333334E-2</v>
-          </cell>
-        </row>
-        <row r="15">
-          <cell r="A15">
-            <v>5</v>
-          </cell>
-          <cell r="B15">
-            <v>0.14599999999999999</v>
-          </cell>
-        </row>
-        <row r="16">
-          <cell r="A16">
-            <v>12.5</v>
-          </cell>
-          <cell r="B16">
-            <v>0.254</v>
-          </cell>
-        </row>
-        <row r="17">
-          <cell r="A17">
-            <v>25</v>
-          </cell>
-          <cell r="B17">
-            <v>0.47633333333333333</v>
-          </cell>
-        </row>
-        <row r="18">
-          <cell r="A18">
-            <v>50</v>
-          </cell>
-          <cell r="B18">
-            <v>0.85399999999999998</v>
-          </cell>
-        </row>
-        <row r="19">
-          <cell r="A19">
-            <v>100</v>
-          </cell>
-          <cell r="B19">
-            <v>1.2565</v>
-          </cell>
-        </row>
-        <row r="20">
-          <cell r="A20">
-            <v>100</v>
-          </cell>
-          <cell r="B20">
-            <v>1.2733333333333334</v>
-          </cell>
-        </row>
-        <row r="21">
-          <cell r="A21">
-            <v>100</v>
-          </cell>
-          <cell r="B21">
-            <v>1.2390000000000001</v>
-          </cell>
-        </row>
-        <row r="24">
-          <cell r="B24" t="str">
-            <v>Avg Abs</v>
-          </cell>
-        </row>
-        <row r="25">
-          <cell r="A25">
-            <v>0</v>
-          </cell>
-          <cell r="B25">
-            <v>5.2666666666666667E-2</v>
-          </cell>
-        </row>
-        <row r="26">
-          <cell r="A26">
-            <v>5</v>
-          </cell>
-          <cell r="B26">
-            <v>0.14433333333333334</v>
-          </cell>
-        </row>
-        <row r="27">
-          <cell r="A27">
-            <v>12.5</v>
-          </cell>
-          <cell r="B27">
-            <v>0.3175</v>
-          </cell>
-        </row>
-        <row r="28">
-          <cell r="A28">
-            <v>25</v>
-          </cell>
-          <cell r="B28">
-            <v>0.4415</v>
-          </cell>
-        </row>
-        <row r="29">
-          <cell r="A29">
-            <v>50</v>
-          </cell>
-          <cell r="B29">
-            <v>0.82099999999999995</v>
-          </cell>
-        </row>
-        <row r="30">
-          <cell r="A30">
-            <v>100</v>
-          </cell>
-          <cell r="B30">
-            <v>1.3305</v>
-          </cell>
-        </row>
-        <row r="31">
-          <cell r="A31">
-            <v>100</v>
-          </cell>
-          <cell r="B31">
-            <v>1.3096666666666665</v>
-          </cell>
-        </row>
-        <row r="32">
-          <cell r="A32">
-            <v>100</v>
-          </cell>
-          <cell r="B32">
-            <v>1.3163333333333334</v>
-          </cell>
-        </row>
-        <row r="35">
-          <cell r="B35" t="str">
-            <v>Avg Abs</v>
-          </cell>
-        </row>
-        <row r="36">
-          <cell r="A36">
-            <v>0</v>
-          </cell>
-          <cell r="B36">
-            <v>5.1666666666666666E-2</v>
-          </cell>
-        </row>
-        <row r="37">
-          <cell r="A37">
-            <v>5</v>
-          </cell>
-          <cell r="B37">
-            <v>0.128</v>
-          </cell>
-        </row>
-        <row r="38">
-          <cell r="A38">
-            <v>12.5</v>
-          </cell>
-          <cell r="B38">
-            <v>0.33766666666666662</v>
-          </cell>
-        </row>
-        <row r="39">
-          <cell r="A39">
-            <v>25</v>
-          </cell>
-          <cell r="B39">
-            <v>0.52849999999999997</v>
-          </cell>
-        </row>
-        <row r="40">
-          <cell r="A40">
-            <v>50</v>
-          </cell>
-          <cell r="B40">
-            <v>0.80149999999999999</v>
-          </cell>
-        </row>
-        <row r="41">
-          <cell r="A41">
-            <v>100</v>
-          </cell>
-          <cell r="B41">
-            <v>1.3576666666666668</v>
-          </cell>
-        </row>
-        <row r="42">
-          <cell r="A42">
-            <v>100</v>
-          </cell>
-          <cell r="B42">
-            <v>1.3259999999999998</v>
-          </cell>
-        </row>
-        <row r="43">
-          <cell r="A43">
-            <v>100</v>
-          </cell>
-          <cell r="B43">
-            <v>1.3109999999999999</v>
-          </cell>
-        </row>
-        <row r="46">
-          <cell r="B46" t="str">
-            <v>Avg Abs</v>
-          </cell>
-        </row>
-        <row r="47">
-          <cell r="A47">
-            <v>0</v>
-          </cell>
-          <cell r="B47">
-            <v>4.9666666666666665E-2</v>
-          </cell>
-        </row>
-        <row r="48">
-          <cell r="A48">
-            <v>5</v>
-          </cell>
-          <cell r="B48">
-            <v>0.13666666666666669</v>
-          </cell>
-        </row>
-        <row r="49">
-          <cell r="A49">
-            <v>12.5</v>
-          </cell>
-          <cell r="B49">
-            <v>0.26533333333333331</v>
-          </cell>
-        </row>
-        <row r="50">
-          <cell r="A50">
-            <v>25</v>
-          </cell>
-          <cell r="B50">
-            <v>0.46599999999999997</v>
-          </cell>
-        </row>
-        <row r="51">
-          <cell r="A51">
-            <v>50</v>
-          </cell>
-          <cell r="B51">
-            <v>0.85599999999999998</v>
-          </cell>
-        </row>
-        <row r="52">
-          <cell r="A52">
-            <v>100</v>
-          </cell>
-          <cell r="B52">
-            <v>1.3816666666666666</v>
-          </cell>
-        </row>
-        <row r="53">
-          <cell r="A53">
-            <v>100</v>
-          </cell>
-          <cell r="B53">
-            <v>1.3360000000000001</v>
-          </cell>
-        </row>
-        <row r="54">
-          <cell r="A54">
-            <v>100</v>
-          </cell>
-          <cell r="B54">
-            <v>1.4139999999999999</v>
-          </cell>
-        </row>
-        <row r="57">
-          <cell r="B57" t="str">
-            <v>Avg Abs</v>
-          </cell>
-        </row>
-        <row r="58">
-          <cell r="A58">
-            <v>0</v>
-          </cell>
-          <cell r="B58">
-            <v>5.1333333333333335E-2</v>
-          </cell>
-        </row>
-        <row r="59">
-          <cell r="A59">
-            <v>5</v>
-          </cell>
-          <cell r="B59">
-            <v>0.13766666666666669</v>
-          </cell>
-        </row>
-        <row r="60">
-          <cell r="A60">
-            <v>12.5</v>
-          </cell>
-          <cell r="B60">
-            <v>0.28466666666666668</v>
-          </cell>
-        </row>
-        <row r="61">
-          <cell r="A61">
-            <v>25</v>
-          </cell>
-          <cell r="B61">
-            <v>0.47599999999999998</v>
-          </cell>
-        </row>
-        <row r="62">
-          <cell r="A62">
-            <v>50</v>
-          </cell>
-          <cell r="B62">
-            <v>0.86099999999999999</v>
-          </cell>
-        </row>
-        <row r="63">
-          <cell r="A63">
-            <v>100</v>
-          </cell>
-          <cell r="B63">
-            <v>1.4079999999999999</v>
-          </cell>
-        </row>
-        <row r="69">
-          <cell r="B69" t="str">
-            <v>Avg Abs</v>
-          </cell>
-        </row>
-        <row r="70">
-          <cell r="A70">
-            <v>0</v>
-          </cell>
-          <cell r="B70">
-            <v>5.1333333333333335E-2</v>
-          </cell>
-        </row>
-        <row r="71">
-          <cell r="A71">
-            <v>5</v>
-          </cell>
-          <cell r="B71">
-            <v>0.127</v>
-          </cell>
-        </row>
-        <row r="72">
-          <cell r="A72">
-            <v>12.5</v>
-          </cell>
-          <cell r="B72">
-            <v>0.30933333333333335</v>
-          </cell>
-        </row>
-        <row r="73">
-          <cell r="A73">
-            <v>25</v>
-          </cell>
-          <cell r="B73">
-            <v>0.50150000000000006</v>
-          </cell>
-        </row>
-        <row r="74">
-          <cell r="A74">
-            <v>50</v>
-          </cell>
-          <cell r="B74">
-            <v>0.86499999999999999</v>
-          </cell>
-        </row>
-        <row r="75">
-          <cell r="A75">
-            <v>100</v>
-          </cell>
-          <cell r="B75">
-            <v>1.405</v>
-          </cell>
-        </row>
-        <row r="80">
-          <cell r="B80" t="str">
-            <v>Avg Abs</v>
-          </cell>
-        </row>
-        <row r="81">
-          <cell r="A81">
-            <v>0</v>
-          </cell>
-          <cell r="B81">
-            <v>5.1000000000000011E-2</v>
-          </cell>
-        </row>
-        <row r="82">
-          <cell r="A82">
-            <v>5</v>
-          </cell>
-          <cell r="B82">
-            <v>0.13933333333333334</v>
-          </cell>
-        </row>
-        <row r="83">
-          <cell r="A83">
-            <v>12.5</v>
-          </cell>
-          <cell r="B83">
-            <v>0.29633333333333334</v>
-          </cell>
-        </row>
-        <row r="84">
-          <cell r="A84">
-            <v>25</v>
-          </cell>
-          <cell r="B84">
-            <v>0.49299999999999999</v>
-          </cell>
-        </row>
-        <row r="85">
-          <cell r="A85">
-            <v>50</v>
-          </cell>
-          <cell r="B85">
-            <v>0.85033333333333339</v>
-          </cell>
-        </row>
-        <row r="86">
-          <cell r="A86">
-            <v>100</v>
-          </cell>
-          <cell r="B86">
-            <v>1.33</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="1" refreshError="1"/>
-      <sheetData sheetId="2" refreshError="1"/>
-      <sheetData sheetId="3" refreshError="1"/>
-      <sheetData sheetId="4" refreshError="1"/>
-      <sheetData sheetId="5" refreshError="1"/>
-      <sheetData sheetId="6" refreshError="1"/>
-      <sheetData sheetId="7" refreshError="1"/>
-      <sheetData sheetId="8" refreshError="1"/>
-      <sheetData sheetId="9" refreshError="1"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -7714,7 +7338,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -7820,7 +7444,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -7962,7 +7586,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -9631,15 +9255,33 @@
       <c r="D12" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="E12" s="6"/>
-      <c r="F12" s="6"/>
-      <c r="G12" s="6"/>
-      <c r="H12" s="6"/>
-      <c r="I12" s="6"/>
-      <c r="J12" s="6"/>
-      <c r="K12" s="6"/>
-      <c r="L12" s="6"/>
-      <c r="M12" s="6"/>
+      <c r="E12" t="s">
+        <v>30</v>
+      </c>
+      <c r="F12" t="s">
+        <v>30</v>
+      </c>
+      <c r="G12" t="s">
+        <v>30</v>
+      </c>
+      <c r="H12" t="s">
+        <v>38</v>
+      </c>
+      <c r="I12" t="s">
+        <v>38</v>
+      </c>
+      <c r="J12" t="s">
+        <v>38</v>
+      </c>
+      <c r="K12" t="s">
+        <v>46</v>
+      </c>
+      <c r="L12" t="s">
+        <v>46</v>
+      </c>
+      <c r="M12" t="s">
+        <v>46</v>
+      </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
@@ -9654,15 +9296,33 @@
       <c r="D13" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="E13" s="6"/>
-      <c r="F13" s="6"/>
-      <c r="G13" s="6"/>
-      <c r="H13" s="6"/>
-      <c r="I13" s="6"/>
-      <c r="J13" s="6"/>
-      <c r="K13" s="6"/>
-      <c r="L13" s="6"/>
-      <c r="M13" s="6"/>
+      <c r="E13" t="s">
+        <v>31</v>
+      </c>
+      <c r="F13" t="s">
+        <v>31</v>
+      </c>
+      <c r="G13" t="s">
+        <v>31</v>
+      </c>
+      <c r="H13" t="s">
+        <v>39</v>
+      </c>
+      <c r="I13" t="s">
+        <v>39</v>
+      </c>
+      <c r="J13" t="s">
+        <v>39</v>
+      </c>
+      <c r="K13" t="s">
+        <v>47</v>
+      </c>
+      <c r="L13" t="s">
+        <v>47</v>
+      </c>
+      <c r="M13" t="s">
+        <v>47</v>
+      </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
@@ -9677,15 +9337,33 @@
       <c r="D14" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="E14" s="6"/>
-      <c r="F14" s="6"/>
-      <c r="G14" s="6"/>
-      <c r="H14" s="6"/>
-      <c r="I14" s="6"/>
-      <c r="J14" s="6"/>
-      <c r="K14" s="6"/>
-      <c r="L14" s="6"/>
-      <c r="M14" s="6"/>
+      <c r="E14" t="s">
+        <v>32</v>
+      </c>
+      <c r="F14" t="s">
+        <v>32</v>
+      </c>
+      <c r="G14" t="s">
+        <v>32</v>
+      </c>
+      <c r="H14" t="s">
+        <v>40</v>
+      </c>
+      <c r="I14" t="s">
+        <v>40</v>
+      </c>
+      <c r="J14" t="s">
+        <v>40</v>
+      </c>
+      <c r="K14" t="s">
+        <v>48</v>
+      </c>
+      <c r="L14" t="s">
+        <v>48</v>
+      </c>
+      <c r="M14" t="s">
+        <v>48</v>
+      </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
@@ -9700,15 +9378,33 @@
       <c r="D15" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="E15" s="6"/>
-      <c r="F15" s="6"/>
-      <c r="G15" s="6"/>
-      <c r="H15" s="6"/>
-      <c r="I15" s="6"/>
-      <c r="J15" s="6"/>
-      <c r="K15" s="6"/>
-      <c r="L15" s="6"/>
-      <c r="M15" s="6"/>
+      <c r="E15" t="s">
+        <v>33</v>
+      </c>
+      <c r="F15" t="s">
+        <v>33</v>
+      </c>
+      <c r="G15" t="s">
+        <v>33</v>
+      </c>
+      <c r="H15" t="s">
+        <v>41</v>
+      </c>
+      <c r="I15" t="s">
+        <v>41</v>
+      </c>
+      <c r="J15" t="s">
+        <v>41</v>
+      </c>
+      <c r="K15" t="s">
+        <v>49</v>
+      </c>
+      <c r="L15" t="s">
+        <v>49</v>
+      </c>
+      <c r="M15" t="s">
+        <v>49</v>
+      </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
@@ -9723,15 +9419,33 @@
       <c r="D16" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="E16" s="6"/>
-      <c r="F16" s="6"/>
-      <c r="G16" s="6"/>
-      <c r="H16" s="6"/>
-      <c r="I16" s="6"/>
-      <c r="J16" s="6"/>
-      <c r="K16" s="6"/>
-      <c r="L16" s="6"/>
-      <c r="M16" s="6"/>
+      <c r="E16" t="s">
+        <v>34</v>
+      </c>
+      <c r="F16" t="s">
+        <v>34</v>
+      </c>
+      <c r="G16" t="s">
+        <v>34</v>
+      </c>
+      <c r="H16" t="s">
+        <v>42</v>
+      </c>
+      <c r="I16" t="s">
+        <v>42</v>
+      </c>
+      <c r="J16" t="s">
+        <v>42</v>
+      </c>
+      <c r="K16" t="s">
+        <v>50</v>
+      </c>
+      <c r="L16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M16" t="s">
+        <v>50</v>
+      </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
@@ -9746,15 +9460,33 @@
       <c r="D17" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="E17" s="6"/>
-      <c r="F17" s="6"/>
-      <c r="G17" s="6"/>
-      <c r="H17" s="6"/>
-      <c r="I17" s="6"/>
-      <c r="J17" s="6"/>
-      <c r="K17" s="6"/>
-      <c r="L17" s="6"/>
-      <c r="M17" s="6"/>
+      <c r="E17" t="s">
+        <v>35</v>
+      </c>
+      <c r="F17" t="s">
+        <v>35</v>
+      </c>
+      <c r="G17" t="s">
+        <v>35</v>
+      </c>
+      <c r="H17" t="s">
+        <v>43</v>
+      </c>
+      <c r="I17" t="s">
+        <v>43</v>
+      </c>
+      <c r="J17" t="s">
+        <v>43</v>
+      </c>
+      <c r="K17" t="s">
+        <v>51</v>
+      </c>
+      <c r="L17" t="s">
+        <v>51</v>
+      </c>
+      <c r="M17" t="s">
+        <v>51</v>
+      </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
@@ -9769,15 +9501,33 @@
       <c r="D18" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="E18" s="6"/>
-      <c r="F18" s="6"/>
-      <c r="G18" s="6"/>
-      <c r="H18" s="6"/>
-      <c r="I18" s="6"/>
-      <c r="J18" s="6"/>
-      <c r="K18" s="6"/>
-      <c r="L18" s="6"/>
-      <c r="M18" s="6"/>
+      <c r="E18" t="s">
+        <v>36</v>
+      </c>
+      <c r="F18" t="s">
+        <v>36</v>
+      </c>
+      <c r="G18" t="s">
+        <v>36</v>
+      </c>
+      <c r="H18" t="s">
+        <v>44</v>
+      </c>
+      <c r="I18" t="s">
+        <v>44</v>
+      </c>
+      <c r="J18" t="s">
+        <v>44</v>
+      </c>
+      <c r="K18" t="s">
+        <v>52</v>
+      </c>
+      <c r="L18" t="s">
+        <v>52</v>
+      </c>
+      <c r="M18" t="s">
+        <v>52</v>
+      </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
@@ -9792,15 +9542,33 @@
       <c r="D19" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="E19" s="6"/>
-      <c r="F19" s="6"/>
-      <c r="G19" s="6"/>
-      <c r="H19" s="6"/>
-      <c r="I19" s="6"/>
-      <c r="J19" s="6"/>
-      <c r="K19" s="6"/>
-      <c r="L19" s="6"/>
-      <c r="M19" s="6"/>
+      <c r="E19" t="s">
+        <v>37</v>
+      </c>
+      <c r="F19" t="s">
+        <v>37</v>
+      </c>
+      <c r="G19" t="s">
+        <v>37</v>
+      </c>
+      <c r="H19" t="s">
+        <v>45</v>
+      </c>
+      <c r="I19" t="s">
+        <v>45</v>
+      </c>
+      <c r="J19" t="s">
+        <v>45</v>
+      </c>
+      <c r="K19" t="s">
+        <v>53</v>
+      </c>
+      <c r="L19" t="s">
+        <v>53</v>
+      </c>
+      <c r="M19" t="s">
+        <v>53</v>
+      </c>
     </row>
     <row r="21" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
@@ -9856,15 +9624,33 @@
       <c r="D22" s="2">
         <v>1</v>
       </c>
-      <c r="E22" s="2"/>
-      <c r="F22" s="2"/>
-      <c r="G22" s="2"/>
-      <c r="H22" s="2"/>
-      <c r="I22" s="2"/>
-      <c r="J22" s="2"/>
-      <c r="K22" s="2"/>
-      <c r="L22" s="2"/>
-      <c r="M22" s="2"/>
+      <c r="E22" s="2">
+        <v>1</v>
+      </c>
+      <c r="F22" s="2">
+        <v>1</v>
+      </c>
+      <c r="G22" s="2">
+        <v>1</v>
+      </c>
+      <c r="H22" s="2">
+        <v>1</v>
+      </c>
+      <c r="I22" s="2">
+        <v>1</v>
+      </c>
+      <c r="J22" s="2">
+        <v>1</v>
+      </c>
+      <c r="K22" s="2">
+        <v>25</v>
+      </c>
+      <c r="L22" s="2">
+        <v>25</v>
+      </c>
+      <c r="M22" s="2">
+        <v>25</v>
+      </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A23" s="4" t="s">
@@ -9879,15 +9665,33 @@
       <c r="D23" s="2">
         <v>1</v>
       </c>
-      <c r="E23" s="2"/>
-      <c r="F23" s="2"/>
-      <c r="G23" s="2"/>
-      <c r="H23" s="2"/>
-      <c r="I23" s="2"/>
-      <c r="J23" s="2"/>
-      <c r="K23" s="2"/>
-      <c r="L23" s="2"/>
-      <c r="M23" s="2"/>
+      <c r="E23" s="2">
+        <v>1</v>
+      </c>
+      <c r="F23" s="2">
+        <v>1</v>
+      </c>
+      <c r="G23" s="2">
+        <v>1</v>
+      </c>
+      <c r="H23" s="2">
+        <v>25</v>
+      </c>
+      <c r="I23" s="2">
+        <v>25</v>
+      </c>
+      <c r="J23" s="2">
+        <v>25</v>
+      </c>
+      <c r="K23" s="2">
+        <v>25</v>
+      </c>
+      <c r="L23" s="2">
+        <v>25</v>
+      </c>
+      <c r="M23" s="2">
+        <v>25</v>
+      </c>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A24" s="4" t="s">
@@ -9902,15 +9706,33 @@
       <c r="D24" s="2">
         <v>1</v>
       </c>
-      <c r="E24" s="2"/>
-      <c r="F24" s="2"/>
-      <c r="G24" s="2"/>
-      <c r="H24" s="2"/>
-      <c r="I24" s="2"/>
-      <c r="J24" s="2"/>
-      <c r="K24" s="2"/>
-      <c r="L24" s="2"/>
-      <c r="M24" s="2"/>
+      <c r="E24" s="2">
+        <v>1</v>
+      </c>
+      <c r="F24" s="2">
+        <v>1</v>
+      </c>
+      <c r="G24" s="2">
+        <v>1</v>
+      </c>
+      <c r="H24" s="2">
+        <v>25</v>
+      </c>
+      <c r="I24" s="2">
+        <v>25</v>
+      </c>
+      <c r="J24" s="2">
+        <v>25</v>
+      </c>
+      <c r="K24" s="2">
+        <v>25</v>
+      </c>
+      <c r="L24" s="2">
+        <v>25</v>
+      </c>
+      <c r="M24" s="2">
+        <v>25</v>
+      </c>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A25" s="4" t="s">
@@ -9925,15 +9747,33 @@
       <c r="D25" s="2">
         <v>1</v>
       </c>
-      <c r="E25" s="2"/>
-      <c r="F25" s="2"/>
-      <c r="G25" s="2"/>
-      <c r="H25" s="2"/>
-      <c r="I25" s="2"/>
-      <c r="J25" s="2"/>
-      <c r="K25" s="2"/>
-      <c r="L25" s="2"/>
-      <c r="M25" s="2"/>
+      <c r="E25" s="2">
+        <v>1</v>
+      </c>
+      <c r="F25" s="2">
+        <v>1</v>
+      </c>
+      <c r="G25" s="2">
+        <v>1</v>
+      </c>
+      <c r="H25" s="2">
+        <v>25</v>
+      </c>
+      <c r="I25" s="2">
+        <v>25</v>
+      </c>
+      <c r="J25" s="2">
+        <v>25</v>
+      </c>
+      <c r="K25" s="2">
+        <v>25</v>
+      </c>
+      <c r="L25" s="2">
+        <v>25</v>
+      </c>
+      <c r="M25" s="2">
+        <v>25</v>
+      </c>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A26" s="4" t="s">
@@ -9948,15 +9788,33 @@
       <c r="D26" s="2">
         <v>1</v>
       </c>
-      <c r="E26" s="2"/>
-      <c r="F26" s="2"/>
-      <c r="G26" s="2"/>
-      <c r="H26" s="2"/>
-      <c r="I26" s="2"/>
-      <c r="J26" s="2"/>
-      <c r="K26" s="2"/>
-      <c r="L26" s="2"/>
-      <c r="M26" s="2"/>
+      <c r="E26" s="2">
+        <v>1</v>
+      </c>
+      <c r="F26" s="2">
+        <v>1</v>
+      </c>
+      <c r="G26" s="2">
+        <v>1</v>
+      </c>
+      <c r="H26" s="2">
+        <v>25</v>
+      </c>
+      <c r="I26" s="2">
+        <v>25</v>
+      </c>
+      <c r="J26" s="2">
+        <v>25</v>
+      </c>
+      <c r="K26" s="2">
+        <v>1</v>
+      </c>
+      <c r="L26" s="2">
+        <v>1</v>
+      </c>
+      <c r="M26" s="2">
+        <v>1</v>
+      </c>
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A27" s="4" t="s">
@@ -9971,15 +9829,33 @@
       <c r="D27" s="2">
         <v>1</v>
       </c>
-      <c r="E27" s="2"/>
-      <c r="F27" s="2"/>
-      <c r="G27" s="2"/>
-      <c r="H27" s="2"/>
-      <c r="I27" s="2"/>
-      <c r="J27" s="2"/>
-      <c r="K27" s="2"/>
-      <c r="L27" s="2"/>
-      <c r="M27" s="2"/>
+      <c r="E27" s="2">
+        <v>1</v>
+      </c>
+      <c r="F27" s="2">
+        <v>1</v>
+      </c>
+      <c r="G27" s="2">
+        <v>1</v>
+      </c>
+      <c r="H27" s="2">
+        <v>25</v>
+      </c>
+      <c r="I27" s="2">
+        <v>25</v>
+      </c>
+      <c r="J27" s="2">
+        <v>25</v>
+      </c>
+      <c r="K27" s="2">
+        <v>1</v>
+      </c>
+      <c r="L27" s="2">
+        <v>1</v>
+      </c>
+      <c r="M27" s="2">
+        <v>1</v>
+      </c>
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A28" s="4" t="s">
@@ -9994,15 +9870,33 @@
       <c r="D28" s="2">
         <v>1</v>
       </c>
-      <c r="E28" s="2"/>
-      <c r="F28" s="2"/>
-      <c r="G28" s="2"/>
-      <c r="H28" s="2"/>
-      <c r="I28" s="2"/>
-      <c r="J28" s="2"/>
-      <c r="K28" s="2"/>
-      <c r="L28" s="2"/>
-      <c r="M28" s="2"/>
+      <c r="E28" s="2">
+        <v>1</v>
+      </c>
+      <c r="F28" s="2">
+        <v>1</v>
+      </c>
+      <c r="G28" s="2">
+        <v>1</v>
+      </c>
+      <c r="H28" s="2">
+        <v>25</v>
+      </c>
+      <c r="I28" s="2">
+        <v>25</v>
+      </c>
+      <c r="J28" s="2">
+        <v>25</v>
+      </c>
+      <c r="K28" s="2">
+        <v>1</v>
+      </c>
+      <c r="L28" s="2">
+        <v>1</v>
+      </c>
+      <c r="M28" s="2">
+        <v>1</v>
+      </c>
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A29" s="4" t="s">
@@ -10017,15 +9911,33 @@
       <c r="D29" s="2">
         <v>1</v>
       </c>
-      <c r="E29" s="2"/>
-      <c r="F29" s="2"/>
-      <c r="G29" s="2"/>
-      <c r="H29" s="2"/>
-      <c r="I29" s="2"/>
-      <c r="J29" s="2"/>
-      <c r="K29" s="2"/>
-      <c r="L29" s="2"/>
-      <c r="M29" s="2"/>
+      <c r="E29" s="2">
+        <v>1</v>
+      </c>
+      <c r="F29" s="2">
+        <v>1</v>
+      </c>
+      <c r="G29" s="2">
+        <v>1</v>
+      </c>
+      <c r="H29" s="2">
+        <v>25</v>
+      </c>
+      <c r="I29" s="2">
+        <v>25</v>
+      </c>
+      <c r="J29" s="2">
+        <v>25</v>
+      </c>
+      <c r="K29" s="2">
+        <v>1</v>
+      </c>
+      <c r="L29" s="2">
+        <v>1</v>
+      </c>
+      <c r="M29" s="2">
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -10459,15 +10371,33 @@
       <c r="D12" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="E12" s="6"/>
-      <c r="F12" s="6"/>
-      <c r="G12" s="6"/>
-      <c r="H12" s="6"/>
-      <c r="I12" s="6"/>
-      <c r="J12" s="6"/>
-      <c r="K12" s="6"/>
-      <c r="L12" s="6"/>
-      <c r="M12" s="6"/>
+      <c r="E12" t="s">
+        <v>54</v>
+      </c>
+      <c r="F12" t="s">
+        <v>54</v>
+      </c>
+      <c r="G12" t="s">
+        <v>54</v>
+      </c>
+      <c r="H12" t="s">
+        <v>62</v>
+      </c>
+      <c r="I12" t="s">
+        <v>62</v>
+      </c>
+      <c r="J12" t="s">
+        <v>62</v>
+      </c>
+      <c r="K12" t="s">
+        <v>70</v>
+      </c>
+      <c r="L12" t="s">
+        <v>70</v>
+      </c>
+      <c r="M12" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
@@ -10482,15 +10412,33 @@
       <c r="D13" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="E13" s="6"/>
-      <c r="F13" s="6"/>
-      <c r="G13" s="6"/>
-      <c r="H13" s="6"/>
-      <c r="I13" s="6"/>
-      <c r="J13" s="6"/>
-      <c r="K13" s="6"/>
-      <c r="L13" s="6"/>
-      <c r="M13" s="6"/>
+      <c r="E13" t="s">
+        <v>55</v>
+      </c>
+      <c r="F13" t="s">
+        <v>55</v>
+      </c>
+      <c r="G13" t="s">
+        <v>55</v>
+      </c>
+      <c r="H13" t="s">
+        <v>63</v>
+      </c>
+      <c r="I13" t="s">
+        <v>63</v>
+      </c>
+      <c r="J13" t="s">
+        <v>63</v>
+      </c>
+      <c r="K13" t="s">
+        <v>73</v>
+      </c>
+      <c r="L13" t="s">
+        <v>73</v>
+      </c>
+      <c r="M13" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
@@ -10505,15 +10453,33 @@
       <c r="D14" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="E14" s="6"/>
-      <c r="F14" s="6"/>
-      <c r="G14" s="6"/>
-      <c r="H14" s="6"/>
-      <c r="I14" s="6"/>
-      <c r="J14" s="6"/>
-      <c r="K14" s="6"/>
-      <c r="L14" s="6"/>
-      <c r="M14" s="6"/>
+      <c r="E14" t="s">
+        <v>56</v>
+      </c>
+      <c r="F14" t="s">
+        <v>56</v>
+      </c>
+      <c r="G14" t="s">
+        <v>56</v>
+      </c>
+      <c r="H14" t="s">
+        <v>64</v>
+      </c>
+      <c r="I14" t="s">
+        <v>64</v>
+      </c>
+      <c r="J14" t="s">
+        <v>64</v>
+      </c>
+      <c r="K14" t="s">
+        <v>74</v>
+      </c>
+      <c r="L14" t="s">
+        <v>74</v>
+      </c>
+      <c r="M14" t="s">
+        <v>74</v>
+      </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
@@ -10528,15 +10494,33 @@
       <c r="D15" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="E15" s="6"/>
-      <c r="F15" s="6"/>
-      <c r="G15" s="6"/>
-      <c r="H15" s="6"/>
-      <c r="I15" s="6"/>
-      <c r="J15" s="6"/>
-      <c r="K15" s="6"/>
-      <c r="L15" s="6"/>
-      <c r="M15" s="6"/>
+      <c r="E15" t="s">
+        <v>57</v>
+      </c>
+      <c r="F15" t="s">
+        <v>57</v>
+      </c>
+      <c r="G15" t="s">
+        <v>57</v>
+      </c>
+      <c r="H15" t="s">
+        <v>65</v>
+      </c>
+      <c r="I15" t="s">
+        <v>65</v>
+      </c>
+      <c r="J15" t="s">
+        <v>65</v>
+      </c>
+      <c r="K15" t="s">
+        <v>75</v>
+      </c>
+      <c r="L15" t="s">
+        <v>75</v>
+      </c>
+      <c r="M15" t="s">
+        <v>75</v>
+      </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
@@ -10551,15 +10535,33 @@
       <c r="D16" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="E16" s="6"/>
-      <c r="F16" s="6"/>
-      <c r="G16" s="6"/>
-      <c r="H16" s="6"/>
-      <c r="I16" s="6"/>
-      <c r="J16" s="6"/>
-      <c r="K16" s="6"/>
-      <c r="L16" s="6"/>
-      <c r="M16" s="6"/>
+      <c r="E16" t="s">
+        <v>58</v>
+      </c>
+      <c r="F16" t="s">
+        <v>58</v>
+      </c>
+      <c r="G16" t="s">
+        <v>58</v>
+      </c>
+      <c r="H16" t="s">
+        <v>66</v>
+      </c>
+      <c r="I16" t="s">
+        <v>66</v>
+      </c>
+      <c r="J16" t="s">
+        <v>66</v>
+      </c>
+      <c r="K16" t="s">
+        <v>76</v>
+      </c>
+      <c r="L16" t="s">
+        <v>76</v>
+      </c>
+      <c r="M16" t="s">
+        <v>76</v>
+      </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
@@ -10574,15 +10576,33 @@
       <c r="D17" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="E17" s="6"/>
-      <c r="F17" s="6"/>
-      <c r="G17" s="6"/>
-      <c r="H17" s="6"/>
-      <c r="I17" s="6"/>
-      <c r="J17" s="6"/>
-      <c r="K17" s="6"/>
-      <c r="L17" s="6"/>
-      <c r="M17" s="6"/>
+      <c r="E17" t="s">
+        <v>59</v>
+      </c>
+      <c r="F17" t="s">
+        <v>59</v>
+      </c>
+      <c r="G17" t="s">
+        <v>59</v>
+      </c>
+      <c r="H17" t="s">
+        <v>67</v>
+      </c>
+      <c r="I17" t="s">
+        <v>67</v>
+      </c>
+      <c r="J17" t="s">
+        <v>67</v>
+      </c>
+      <c r="K17" t="s">
+        <v>71</v>
+      </c>
+      <c r="L17" t="s">
+        <v>71</v>
+      </c>
+      <c r="M17" t="s">
+        <v>71</v>
+      </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
@@ -10597,15 +10617,33 @@
       <c r="D18" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="E18" s="6"/>
-      <c r="F18" s="6"/>
-      <c r="G18" s="6"/>
-      <c r="H18" s="6"/>
-      <c r="I18" s="6"/>
-      <c r="J18" s="6"/>
-      <c r="K18" s="6"/>
-      <c r="L18" s="6"/>
-      <c r="M18" s="6"/>
+      <c r="E18" t="s">
+        <v>60</v>
+      </c>
+      <c r="F18" t="s">
+        <v>60</v>
+      </c>
+      <c r="G18" t="s">
+        <v>60</v>
+      </c>
+      <c r="H18" t="s">
+        <v>68</v>
+      </c>
+      <c r="I18" t="s">
+        <v>68</v>
+      </c>
+      <c r="J18" t="s">
+        <v>68</v>
+      </c>
+      <c r="K18" t="s">
+        <v>72</v>
+      </c>
+      <c r="L18" t="s">
+        <v>72</v>
+      </c>
+      <c r="M18" t="s">
+        <v>72</v>
+      </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
@@ -10620,15 +10658,33 @@
       <c r="D19" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="E19" s="6"/>
-      <c r="F19" s="6"/>
-      <c r="G19" s="6"/>
-      <c r="H19" s="6"/>
-      <c r="I19" s="6"/>
-      <c r="J19" s="6"/>
-      <c r="K19" s="6"/>
-      <c r="L19" s="6"/>
-      <c r="M19" s="6"/>
+      <c r="E19" t="s">
+        <v>61</v>
+      </c>
+      <c r="F19" t="s">
+        <v>61</v>
+      </c>
+      <c r="G19" t="s">
+        <v>61</v>
+      </c>
+      <c r="H19" t="s">
+        <v>69</v>
+      </c>
+      <c r="I19" t="s">
+        <v>69</v>
+      </c>
+      <c r="J19" t="s">
+        <v>69</v>
+      </c>
+      <c r="K19" t="s">
+        <v>77</v>
+      </c>
+      <c r="L19" t="s">
+        <v>77</v>
+      </c>
+      <c r="M19" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="21" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
@@ -10684,15 +10740,33 @@
       <c r="D22" s="2">
         <v>1</v>
       </c>
-      <c r="E22" s="2"/>
-      <c r="F22" s="2"/>
-      <c r="G22" s="2"/>
-      <c r="H22" s="2"/>
-      <c r="I22" s="2"/>
-      <c r="J22" s="2"/>
-      <c r="K22" s="2"/>
-      <c r="L22" s="2"/>
-      <c r="M22" s="2"/>
+      <c r="E22" s="2">
+        <v>1</v>
+      </c>
+      <c r="F22" s="2">
+        <v>1</v>
+      </c>
+      <c r="G22" s="2">
+        <v>1</v>
+      </c>
+      <c r="H22" s="2">
+        <v>1</v>
+      </c>
+      <c r="I22" s="2">
+        <v>1</v>
+      </c>
+      <c r="J22" s="2">
+        <v>1</v>
+      </c>
+      <c r="K22" s="2">
+        <v>25</v>
+      </c>
+      <c r="L22" s="2">
+        <v>25</v>
+      </c>
+      <c r="M22" s="2">
+        <v>25</v>
+      </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A23" s="4" t="s">
@@ -10707,15 +10781,33 @@
       <c r="D23" s="2">
         <v>1</v>
       </c>
-      <c r="E23" s="2"/>
-      <c r="F23" s="2"/>
-      <c r="G23" s="2"/>
-      <c r="H23" s="2"/>
-      <c r="I23" s="2"/>
-      <c r="J23" s="2"/>
-      <c r="K23" s="2"/>
-      <c r="L23" s="2"/>
-      <c r="M23" s="2"/>
+      <c r="E23" s="2">
+        <v>1</v>
+      </c>
+      <c r="F23" s="2">
+        <v>1</v>
+      </c>
+      <c r="G23" s="2">
+        <v>1</v>
+      </c>
+      <c r="H23" s="2">
+        <v>1</v>
+      </c>
+      <c r="I23" s="2">
+        <v>1</v>
+      </c>
+      <c r="J23" s="2">
+        <v>1</v>
+      </c>
+      <c r="K23" s="2">
+        <v>25</v>
+      </c>
+      <c r="L23" s="2">
+        <v>25</v>
+      </c>
+      <c r="M23" s="2">
+        <v>25</v>
+      </c>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A24" s="4" t="s">
@@ -10730,15 +10822,33 @@
       <c r="D24" s="2">
         <v>1</v>
       </c>
-      <c r="E24" s="2"/>
-      <c r="F24" s="2"/>
-      <c r="G24" s="2"/>
-      <c r="H24" s="2"/>
-      <c r="I24" s="2"/>
-      <c r="J24" s="2"/>
-      <c r="K24" s="2"/>
-      <c r="L24" s="2"/>
-      <c r="M24" s="2"/>
+      <c r="E24" s="2">
+        <v>1</v>
+      </c>
+      <c r="F24" s="2">
+        <v>1</v>
+      </c>
+      <c r="G24" s="2">
+        <v>1</v>
+      </c>
+      <c r="H24" s="2">
+        <v>1</v>
+      </c>
+      <c r="I24" s="2">
+        <v>1</v>
+      </c>
+      <c r="J24" s="2">
+        <v>1</v>
+      </c>
+      <c r="K24" s="2">
+        <v>1</v>
+      </c>
+      <c r="L24" s="2">
+        <v>1</v>
+      </c>
+      <c r="M24" s="2">
+        <v>1</v>
+      </c>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A25" s="4" t="s">
@@ -10753,15 +10863,33 @@
       <c r="D25" s="2">
         <v>1</v>
       </c>
-      <c r="E25" s="2"/>
-      <c r="F25" s="2"/>
-      <c r="G25" s="2"/>
-      <c r="H25" s="2"/>
-      <c r="I25" s="2"/>
-      <c r="J25" s="2"/>
-      <c r="K25" s="2"/>
-      <c r="L25" s="2"/>
-      <c r="M25" s="2"/>
+      <c r="E25" s="2">
+        <v>1</v>
+      </c>
+      <c r="F25" s="2">
+        <v>1</v>
+      </c>
+      <c r="G25" s="2">
+        <v>1</v>
+      </c>
+      <c r="H25" s="2">
+        <v>1</v>
+      </c>
+      <c r="I25" s="2">
+        <v>1</v>
+      </c>
+      <c r="J25" s="2">
+        <v>1</v>
+      </c>
+      <c r="K25" s="2">
+        <v>25</v>
+      </c>
+      <c r="L25" s="2">
+        <v>25</v>
+      </c>
+      <c r="M25" s="2">
+        <v>25</v>
+      </c>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A26" s="4" t="s">
@@ -10776,15 +10904,33 @@
       <c r="D26" s="2">
         <v>1</v>
       </c>
-      <c r="E26" s="2"/>
-      <c r="F26" s="2"/>
-      <c r="G26" s="2"/>
-      <c r="H26" s="2"/>
-      <c r="I26" s="2"/>
-      <c r="J26" s="2"/>
-      <c r="K26" s="2"/>
-      <c r="L26" s="2"/>
-      <c r="M26" s="2"/>
+      <c r="E26" s="2">
+        <v>1</v>
+      </c>
+      <c r="F26" s="2">
+        <v>1</v>
+      </c>
+      <c r="G26" s="2">
+        <v>1</v>
+      </c>
+      <c r="H26" s="2">
+        <v>1</v>
+      </c>
+      <c r="I26" s="2">
+        <v>1</v>
+      </c>
+      <c r="J26" s="2">
+        <v>1</v>
+      </c>
+      <c r="K26" s="2">
+        <v>25</v>
+      </c>
+      <c r="L26" s="2">
+        <v>25</v>
+      </c>
+      <c r="M26" s="2">
+        <v>25</v>
+      </c>
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A27" s="4" t="s">
@@ -10799,15 +10945,33 @@
       <c r="D27" s="2">
         <v>1</v>
       </c>
-      <c r="E27" s="2"/>
-      <c r="F27" s="2"/>
-      <c r="G27" s="2"/>
-      <c r="H27" s="2"/>
-      <c r="I27" s="2"/>
-      <c r="J27" s="2"/>
-      <c r="K27" s="2"/>
-      <c r="L27" s="2"/>
-      <c r="M27" s="2"/>
+      <c r="E27" s="2">
+        <v>1</v>
+      </c>
+      <c r="F27" s="2">
+        <v>1</v>
+      </c>
+      <c r="G27" s="2">
+        <v>1</v>
+      </c>
+      <c r="H27" s="2">
+        <v>1</v>
+      </c>
+      <c r="I27" s="2">
+        <v>1</v>
+      </c>
+      <c r="J27" s="2">
+        <v>1</v>
+      </c>
+      <c r="K27" s="2">
+        <v>1</v>
+      </c>
+      <c r="L27" s="2">
+        <v>1</v>
+      </c>
+      <c r="M27" s="2">
+        <v>1</v>
+      </c>
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A28" s="4" t="s">
@@ -10822,15 +10986,33 @@
       <c r="D28" s="2">
         <v>1</v>
       </c>
-      <c r="E28" s="2"/>
-      <c r="F28" s="2"/>
-      <c r="G28" s="2"/>
-      <c r="H28" s="2"/>
-      <c r="I28" s="2"/>
-      <c r="J28" s="2"/>
-      <c r="K28" s="2"/>
-      <c r="L28" s="2"/>
-      <c r="M28" s="2"/>
+      <c r="E28" s="2">
+        <v>1</v>
+      </c>
+      <c r="F28" s="2">
+        <v>1</v>
+      </c>
+      <c r="G28" s="2">
+        <v>1</v>
+      </c>
+      <c r="H28" s="2">
+        <v>1</v>
+      </c>
+      <c r="I28" s="2">
+        <v>1</v>
+      </c>
+      <c r="J28" s="2">
+        <v>1</v>
+      </c>
+      <c r="K28" s="2">
+        <v>25</v>
+      </c>
+      <c r="L28" s="2">
+        <v>25</v>
+      </c>
+      <c r="M28" s="2">
+        <v>25</v>
+      </c>
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A29" s="4" t="s">
@@ -10845,15 +11027,33 @@
       <c r="D29" s="2">
         <v>1</v>
       </c>
-      <c r="E29" s="2"/>
-      <c r="F29" s="2"/>
-      <c r="G29" s="2"/>
-      <c r="H29" s="2"/>
-      <c r="I29" s="2"/>
-      <c r="J29" s="2"/>
-      <c r="K29" s="2"/>
-      <c r="L29" s="2"/>
-      <c r="M29" s="2"/>
+      <c r="E29" s="2">
+        <v>1</v>
+      </c>
+      <c r="F29" s="2">
+        <v>1</v>
+      </c>
+      <c r="G29" s="2">
+        <v>1</v>
+      </c>
+      <c r="H29" s="2">
+        <v>1</v>
+      </c>
+      <c r="I29" s="2">
+        <v>1</v>
+      </c>
+      <c r="J29" s="2">
+        <v>1</v>
+      </c>
+      <c r="K29" s="2">
+        <v>25</v>
+      </c>
+      <c r="L29" s="2">
+        <v>25</v>
+      </c>
+      <c r="M29" s="2">
+        <v>25</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -11287,7 +11487,9 @@
       <c r="D12" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="E12" s="6"/>
+      <c r="E12" t="s">
+        <v>78</v>
+      </c>
       <c r="F12" s="6"/>
       <c r="G12" s="6"/>
       <c r="H12" s="6"/>
@@ -11310,7 +11512,6 @@
       <c r="D13" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="E13" s="6"/>
       <c r="F13" s="6"/>
       <c r="G13" s="6"/>
       <c r="H13" s="6"/>

</xml_diff>